<commit_message>
rename data collection type values: survey→qualitative, telemetry→quantitative
Updated dashboard (chart.js, metrics-selection.js, index.html) and data.json
to reflect the renamed Data Collection Type values from the source Excel file.
The metric detail pop-up label was also corrected from "Qualitative" to "Self-reported".
</commit_message>
<xml_diff>
--- a/metrics and parser/DevEx_Metrics.xlsx
+++ b/metrics and parser/DevEx_Metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\DEV\UZH\DX-Metrics-Compass\metrics and parser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56401978-88B9-47A4-B572-C9EEF46C63CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1977848B-A203-4DB4-B88D-D1732F9C5A3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" tabRatio="506" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2307,16 +2307,16 @@
     <t>Avg. Weekly Focus Time per Engineer; Avg. Number of Days with Sufficient Focus Time; Focus Time and Interruption Metrics; Uninterrupted Focus Time</t>
   </si>
   <si>
-    <t>telemetry</t>
-  </si>
-  <si>
-    <t>survey</t>
-  </si>
-  <si>
     <t>Data Collection Type</t>
   </si>
   <si>
     <t>Aims to capture all active human developer time spent on a particular diff, split by the different roles involved. This information is made available in a privacy-aware manner. Active human work on a computer tends to be highly sequential, even if such individual sequences can be extremely short.</t>
+  </si>
+  <si>
+    <t>qualitative</t>
+  </si>
+  <si>
+    <t>quantitative</t>
   </si>
 </sst>
 </file>
@@ -2393,7 +2393,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -2446,12 +2446,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2464,6 +2458,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2509,16 +2513,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2539,21 +2533,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2639,21 +2633,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3189,31 +3183,31 @@
       <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="20" t="s">
-        <v>737</v>
-      </c>
-      <c r="H1" s="20" t="s">
+      <c r="G1" s="1" t="s">
+        <v>735</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="20" t="s">
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="20" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="20" t="s">
+      <c r="M1" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="N1" s="20" t="s">
+      <c r="N1" s="1" t="s">
         <v>523</v>
       </c>
-      <c r="O1" s="20" t="s">
+      <c r="O1" s="1" t="s">
         <v>525</v>
       </c>
       <c r="P1" s="18" t="s">
@@ -3249,7 +3243,7 @@
         <v>14</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>15</v>
@@ -3314,7 +3308,7 @@
         <v>20</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>21</v>
@@ -3379,7 +3373,7 @@
         <v>24</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>524</v>
@@ -3444,7 +3438,7 @@
         <v>27</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>15</v>
@@ -3509,7 +3503,7 @@
         <v>30</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>524</v>
@@ -3574,7 +3568,7 @@
         <v>33</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>10</v>
@@ -3639,7 +3633,7 @@
         <v>35</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>36</v>
@@ -3704,7 +3698,7 @@
         <v>40</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>36</v>
@@ -3769,7 +3763,7 @@
         <v>43</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>36</v>
@@ -3834,7 +3828,7 @@
         <v>45</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>15</v>
@@ -3899,7 +3893,7 @@
         <v>47</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>36</v>
@@ -3964,7 +3958,7 @@
         <v>51</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>52</v>
@@ -4029,7 +4023,7 @@
         <v>54</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>36</v>
@@ -4094,7 +4088,7 @@
         <v>56</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>57</v>
@@ -4159,7 +4153,7 @@
         <v>60</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>524</v>
@@ -4224,7 +4218,7 @@
         <v>64</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>15</v>
@@ -4289,7 +4283,7 @@
         <v>67</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>52</v>
@@ -4354,7 +4348,7 @@
         <v>71</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>10</v>
@@ -4419,7 +4413,7 @@
         <v>74</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>75</v>
@@ -4484,7 +4478,7 @@
         <v>77</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>75</v>
@@ -4549,7 +4543,7 @@
         <v>78</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>15</v>
@@ -4614,7 +4608,7 @@
         <v>81</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>524</v>
@@ -4679,7 +4673,7 @@
         <v>83</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>36</v>
@@ -4744,7 +4738,7 @@
         <v>85</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>75</v>
@@ -4809,7 +4803,7 @@
         <v>87</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>36</v>
@@ -4874,7 +4868,7 @@
         <v>91</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>75</v>
@@ -4939,7 +4933,7 @@
         <v>93</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>15</v>
@@ -5004,7 +4998,7 @@
         <v>96</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>21</v>
@@ -5069,7 +5063,7 @@
         <v>98</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>524</v>
@@ -5134,7 +5128,7 @@
         <v>101</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>524</v>
@@ -5199,7 +5193,7 @@
         <v>104</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>10</v>
@@ -5261,10 +5255,10 @@
         <v>463</v>
       </c>
       <c r="F33" s="7" t="s">
+        <v>736</v>
+      </c>
+      <c r="G33" s="3" t="s">
         <v>738</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>735</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>15</v>
@@ -5329,7 +5323,7 @@
         <v>107</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>15</v>
@@ -5394,7 +5388,7 @@
         <v>109</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>524</v>
@@ -5459,7 +5453,7 @@
         <v>111</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>524</v>
@@ -5524,7 +5518,7 @@
         <v>113</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>36</v>
@@ -5589,7 +5583,7 @@
         <v>115</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>524</v>
@@ -5654,7 +5648,7 @@
         <v>119</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>21</v>
@@ -5719,7 +5713,7 @@
         <v>122</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>21</v>
@@ -5784,7 +5778,7 @@
         <v>125</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>52</v>
@@ -5849,7 +5843,7 @@
         <v>128</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>524</v>
@@ -5914,7 +5908,7 @@
         <v>130</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>15</v>
@@ -5979,7 +5973,7 @@
         <v>132</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>15</v>
@@ -6044,7 +6038,7 @@
         <v>134</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>524</v>
@@ -6109,7 +6103,7 @@
         <v>137</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H46" s="3" t="s">
         <v>10</v>
@@ -6174,7 +6168,7 @@
         <v>139</v>
       </c>
       <c r="G47" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H47" s="3" t="s">
         <v>524</v>
@@ -6239,7 +6233,7 @@
         <v>141</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H48" s="3" t="s">
         <v>524</v>
@@ -6304,7 +6298,7 @@
         <v>145</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H49" s="3" t="s">
         <v>15</v>
@@ -6369,7 +6363,7 @@
         <v>148</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H50" s="3" t="s">
         <v>36</v>
@@ -6434,7 +6428,7 @@
         <v>150</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>21</v>
@@ -6499,7 +6493,7 @@
         <v>152</v>
       </c>
       <c r="G52" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H52" s="3" t="s">
         <v>21</v>
@@ -6564,7 +6558,7 @@
         <v>154</v>
       </c>
       <c r="G53" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H53" s="3" t="s">
         <v>52</v>
@@ -6629,7 +6623,7 @@
         <v>155</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>52</v>
@@ -6694,7 +6688,7 @@
         <v>157</v>
       </c>
       <c r="G55" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H55" s="3" t="s">
         <v>75</v>
@@ -6759,7 +6753,7 @@
         <v>159</v>
       </c>
       <c r="G56" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H56" s="3" t="s">
         <v>36</v>
@@ -6824,7 +6818,7 @@
         <v>161</v>
       </c>
       <c r="G57" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H57" s="3" t="s">
         <v>15</v>
@@ -6889,7 +6883,7 @@
         <v>163</v>
       </c>
       <c r="G58" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H58" s="3" t="s">
         <v>10</v>
@@ -6954,7 +6948,7 @@
         <v>166</v>
       </c>
       <c r="G59" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H59" s="3" t="s">
         <v>21</v>
@@ -7019,7 +7013,7 @@
         <v>169</v>
       </c>
       <c r="G60" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H60" s="3" t="s">
         <v>10</v>
@@ -7084,7 +7078,7 @@
         <v>171</v>
       </c>
       <c r="G61" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H61" s="3" t="s">
         <v>36</v>
@@ -7149,7 +7143,7 @@
         <v>173</v>
       </c>
       <c r="G62" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H62" s="3" t="s">
         <v>10</v>
@@ -7214,7 +7208,7 @@
         <v>175</v>
       </c>
       <c r="G63" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H63" s="3" t="s">
         <v>524</v>
@@ -7279,7 +7273,7 @@
         <v>178</v>
       </c>
       <c r="G64" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H64" s="3" t="s">
         <v>524</v>
@@ -7344,7 +7338,7 @@
         <v>180</v>
       </c>
       <c r="G65" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H65" s="3" t="s">
         <v>75</v>
@@ -7409,7 +7403,7 @@
         <v>182</v>
       </c>
       <c r="G66" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H66" s="3" t="s">
         <v>75</v>
@@ -7474,7 +7468,7 @@
         <v>184</v>
       </c>
       <c r="G67" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H67" s="3" t="s">
         <v>36</v>
@@ -7539,7 +7533,7 @@
         <v>186</v>
       </c>
       <c r="G68" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H68" s="3" t="s">
         <v>10</v>
@@ -7604,7 +7598,7 @@
         <v>188</v>
       </c>
       <c r="G69" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H69" s="3" t="s">
         <v>524</v>
@@ -7669,7 +7663,7 @@
         <v>189</v>
       </c>
       <c r="G70" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H70" s="3" t="s">
         <v>21</v>
@@ -7734,7 +7728,7 @@
         <v>191</v>
       </c>
       <c r="G71" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H71" s="3" t="s">
         <v>15</v>
@@ -7799,7 +7793,7 @@
         <v>193</v>
       </c>
       <c r="G72" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H72" s="3" t="s">
         <v>15</v>
@@ -7864,7 +7858,7 @@
         <v>195</v>
       </c>
       <c r="G73" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H73" s="3" t="s">
         <v>36</v>
@@ -7929,7 +7923,7 @@
         <v>197</v>
       </c>
       <c r="G74" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H74" s="3" t="s">
         <v>36</v>
@@ -7994,7 +7988,7 @@
         <v>199</v>
       </c>
       <c r="G75" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H75" s="3" t="s">
         <v>36</v>
@@ -8059,7 +8053,7 @@
         <v>201</v>
       </c>
       <c r="G76" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H76" s="3" t="s">
         <v>15</v>
@@ -8124,7 +8118,7 @@
         <v>203</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H77" s="3" t="s">
         <v>52</v>
@@ -8189,7 +8183,7 @@
         <v>205</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H78" s="3" t="s">
         <v>10</v>
@@ -8254,7 +8248,7 @@
         <v>207</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H79" s="3" t="s">
         <v>75</v>
@@ -8319,7 +8313,7 @@
         <v>210</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H80" s="3" t="s">
         <v>21</v>
@@ -8384,7 +8378,7 @@
         <v>212</v>
       </c>
       <c r="G81" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H81" s="3" t="s">
         <v>21</v>
@@ -8449,7 +8443,7 @@
         <v>214</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H82" s="3" t="s">
         <v>10</v>
@@ -8514,7 +8508,7 @@
         <v>216</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H83" s="3" t="s">
         <v>10</v>
@@ -8579,7 +8573,7 @@
         <v>218</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H84" s="3" t="s">
         <v>10</v>
@@ -8644,7 +8638,7 @@
         <v>221</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H85" s="3" t="s">
         <v>15</v>
@@ -8709,7 +8703,7 @@
         <v>224</v>
       </c>
       <c r="G86" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H86" s="3" t="s">
         <v>524</v>
@@ -8774,7 +8768,7 @@
         <v>226</v>
       </c>
       <c r="G87" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H87" s="3" t="s">
         <v>21</v>
@@ -8839,7 +8833,7 @@
         <v>228</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H88" s="3" t="s">
         <v>15</v>
@@ -8904,7 +8898,7 @@
         <v>230</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H89" s="3" t="s">
         <v>15</v>
@@ -8969,7 +8963,7 @@
         <v>232</v>
       </c>
       <c r="G90" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H90" s="3" t="s">
         <v>21</v>
@@ -9034,7 +9028,7 @@
         <v>234</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H91" s="3" t="s">
         <v>524</v>
@@ -9099,7 +9093,7 @@
         <v>237</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H92" s="3" t="s">
         <v>57</v>
@@ -9164,7 +9158,7 @@
         <v>239</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H93" s="3" t="s">
         <v>52</v>
@@ -9229,7 +9223,7 @@
         <v>241</v>
       </c>
       <c r="G94" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H94" s="3" t="s">
         <v>36</v>
@@ -9294,7 +9288,7 @@
         <v>243</v>
       </c>
       <c r="G95" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H95" s="3" t="s">
         <v>36</v>
@@ -9359,7 +9353,7 @@
         <v>245</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H96" s="3" t="s">
         <v>21</v>
@@ -9424,7 +9418,7 @@
         <v>248</v>
       </c>
       <c r="G97" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H97" s="3" t="s">
         <v>15</v>
@@ -9489,7 +9483,7 @@
         <v>250</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H98" s="3" t="s">
         <v>15</v>
@@ -9554,7 +9548,7 @@
         <v>252</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H99" s="3" t="s">
         <v>15</v>
@@ -9619,7 +9613,7 @@
         <v>254</v>
       </c>
       <c r="G100" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H100" s="3" t="s">
         <v>15</v>
@@ -9684,7 +9678,7 @@
         <v>257</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H101" s="3" t="s">
         <v>524</v>
@@ -9749,7 +9743,7 @@
         <v>260</v>
       </c>
       <c r="G102" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H102" s="3" t="s">
         <v>57</v>
@@ -9814,7 +9808,7 @@
         <v>263</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H103" s="3" t="s">
         <v>57</v>
@@ -9879,7 +9873,7 @@
         <v>265</v>
       </c>
       <c r="G104" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H104" s="3" t="s">
         <v>57</v>
@@ -9944,7 +9938,7 @@
         <v>647</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H105" s="3" t="s">
         <v>57</v>
@@ -10009,7 +10003,7 @@
         <v>267</v>
       </c>
       <c r="G106" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H106" s="3" t="s">
         <v>524</v>
@@ -10074,7 +10068,7 @@
         <v>517</v>
       </c>
       <c r="G107" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H107" t="s">
         <v>36</v>
@@ -10139,7 +10133,7 @@
         <v>519</v>
       </c>
       <c r="G108" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H108" t="s">
         <v>524</v>
@@ -10204,7 +10198,7 @@
         <v>520</v>
       </c>
       <c r="G109" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H109" t="s">
         <v>57</v>
@@ -10269,7 +10263,7 @@
         <v>521</v>
       </c>
       <c r="G110" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H110" t="s">
         <v>524</v>
@@ -10334,7 +10328,7 @@
         <v>516</v>
       </c>
       <c r="G111" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H111" t="s">
         <v>10</v>
@@ -10399,7 +10393,7 @@
         <v>570</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>21</v>
@@ -10464,7 +10458,7 @@
         <v>611</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H113" s="3" t="s">
         <v>15</v>
@@ -10529,7 +10523,7 @@
         <v>616</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H114" s="3" t="s">
         <v>57</v>
@@ -10594,7 +10588,7 @@
         <v>619</v>
       </c>
       <c r="G115" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H115" s="3" t="s">
         <v>57</v>
@@ -10659,7 +10653,7 @@
         <v>626</v>
       </c>
       <c r="G116" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H116" s="3" t="s">
         <v>57</v>
@@ -10724,7 +10718,7 @@
         <v>631</v>
       </c>
       <c r="G117" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H117" s="3" t="s">
         <v>15</v>
@@ -10789,7 +10783,7 @@
         <v>632</v>
       </c>
       <c r="G118" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H118" t="s">
         <v>10</v>
@@ -10854,7 +10848,7 @@
         <v>636</v>
       </c>
       <c r="G119" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H119" t="s">
         <v>10</v>
@@ -10919,7 +10913,7 @@
         <v>638</v>
       </c>
       <c r="G120" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H120" s="3" t="s">
         <v>15</v>
@@ -10984,7 +10978,7 @@
         <v>644</v>
       </c>
       <c r="G121" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H121" s="3" t="s">
         <v>10</v>
@@ -11049,7 +11043,7 @@
         <v>655</v>
       </c>
       <c r="G122" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H122" s="3" t="s">
         <v>21</v>
@@ -11114,7 +11108,7 @@
         <v>670</v>
       </c>
       <c r="G123" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H123" s="3" t="s">
         <v>524</v>
@@ -11179,7 +11173,7 @@
         <v>682</v>
       </c>
       <c r="G124" s="3" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="H124" s="3" t="s">
         <v>15</v>
@@ -11244,7 +11238,7 @@
         <v>698</v>
       </c>
       <c r="G125" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H125" s="3" t="s">
         <v>524</v>
@@ -11309,7 +11303,7 @@
         <v>701</v>
       </c>
       <c r="G126" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H126" s="3" t="s">
         <v>524</v>
@@ -11374,7 +11368,7 @@
         <v>706</v>
       </c>
       <c r="G127" s="3" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="H127" s="3" t="s">
         <v>524</v>
@@ -11522,8 +11516,8 @@
     <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F48">
-    <cfRule type="duplicateValues" dxfId="19" priority="20"/>
-    <cfRule type="duplicateValues" dxfId="18" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F73">
     <cfRule type="duplicateValues" dxfId="17" priority="7"/>
@@ -11546,20 +11540,20 @@
     <cfRule type="duplicateValues" dxfId="10" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J47">
-    <cfRule type="duplicateValues" dxfId="9" priority="16"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J64">
     <cfRule type="duplicateValues" dxfId="7" priority="12"/>
     <cfRule type="duplicateValues" dxfId="6" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J69">
-    <cfRule type="duplicateValues" dxfId="5" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J106">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
updated compass to handle metrics that are quantitative and qualitative
</commit_message>
<xml_diff>
--- a/metrics and parser/DevEx_Metrics.xlsx
+++ b/metrics and parser/DevEx_Metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\DEV\UZH\DX-Metrics-Compass\metrics and parser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DD9DB2D-DC22-420E-B101-F5877A0D68F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{092770D1-0B9B-474B-9130-819E1EE4F08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" tabRatio="506" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2378,7 +2378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -2428,12 +2428,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2441,21 +2435,21 @@
   <dxfs count="39">
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2501,16 +2495,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2531,21 +2515,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2631,21 +2615,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2826,6 +2810,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3131,7 +3125,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:S124"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3143,8 +3136,7 @@
     <col min="6" max="6" width="36.5703125" style="3" customWidth="1"/>
     <col min="7" max="7" width="31.7109375" style="3" customWidth="1"/>
     <col min="8" max="9" width="17.85546875" style="3" customWidth="1"/>
-    <col min="10" max="12" width="28.42578125" style="3" customWidth="1"/>
-    <col min="13" max="13" width="28.42578125" style="20" customWidth="1"/>
+    <col min="10" max="13" width="28.42578125" style="3" customWidth="1"/>
     <col min="14" max="15" width="9.140625" style="3"/>
     <col min="16" max="16" width="18.7109375" style="14" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="30.7109375" style="14" customWidth="1"/>
@@ -3190,7 +3182,7 @@
       <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="19" t="s">
+      <c r="M1" s="1" t="s">
         <v>515</v>
       </c>
       <c r="N1" s="1" t="s">
@@ -3212,7 +3204,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2</v>
       </c>
@@ -3277,7 +3269,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>4</v>
       </c>
@@ -3342,7 +3334,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>9</v>
       </c>
@@ -3407,7 +3399,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>10</v>
       </c>
@@ -3472,7 +3464,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>11</v>
       </c>
@@ -3537,7 +3529,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>12</v>
       </c>
@@ -3602,7 +3594,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="165" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="165" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>13</v>
       </c>
@@ -3667,7 +3659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>14</v>
       </c>
@@ -3732,7 +3724,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="150" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="150" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>15</v>
       </c>
@@ -3797,7 +3789,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>16</v>
       </c>
@@ -3862,7 +3854,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>17</v>
       </c>
@@ -3927,7 +3919,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>18</v>
       </c>
@@ -3992,7 +3984,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>19</v>
       </c>
@@ -4057,7 +4049,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>20</v>
       </c>
@@ -4122,7 +4114,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>22</v>
       </c>
@@ -4187,7 +4179,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>23</v>
       </c>
@@ -4252,7 +4244,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="150" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" ht="150" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>24</v>
       </c>
@@ -4317,7 +4309,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>25</v>
       </c>
@@ -4382,7 +4374,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>26</v>
       </c>
@@ -4447,7 +4439,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>27</v>
       </c>
@@ -4512,7 +4504,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>29</v>
       </c>
@@ -4577,7 +4569,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>30</v>
       </c>
@@ -4642,7 +4634,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>31</v>
       </c>
@@ -4707,7 +4699,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>32</v>
       </c>
@@ -4772,7 +4764,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>33</v>
       </c>
@@ -4837,7 +4829,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>34</v>
       </c>
@@ -4902,7 +4894,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>35</v>
       </c>
@@ -4967,7 +4959,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="180" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" ht="180" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>36</v>
       </c>
@@ -5032,7 +5024,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="255" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" ht="255" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>37</v>
       </c>
@@ -5097,7 +5089,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="135" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" ht="135" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>38</v>
       </c>
@@ -5162,7 +5154,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>39</v>
       </c>
@@ -5227,7 +5219,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>40</v>
       </c>
@@ -5292,7 +5284,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>41</v>
       </c>
@@ -5357,7 +5349,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>42</v>
       </c>
@@ -5422,7 +5414,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>43</v>
       </c>
@@ -5487,7 +5479,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>44</v>
       </c>
@@ -5552,7 +5544,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>45</v>
       </c>
@@ -5617,7 +5609,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>46</v>
       </c>
@@ -5722,7 +5714,7 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="M40" s="20">
+      <c r="M40" s="3">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
@@ -5747,7 +5739,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="41" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>51</v>
       </c>
@@ -5812,7 +5804,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>54</v>
       </c>
@@ -5877,7 +5869,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="135" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" ht="135" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>56</v>
       </c>
@@ -5942,7 +5934,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>57</v>
       </c>
@@ -6007,7 +5999,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="360" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" ht="360" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>58</v>
       </c>
@@ -6112,7 +6104,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="M46" s="20">
+      <c r="M46" s="3">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -6137,7 +6129,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>62</v>
       </c>
@@ -6202,7 +6194,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>63</v>
       </c>
@@ -6267,7 +6259,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>64</v>
       </c>
@@ -6332,7 +6324,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="150" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" ht="150" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>65</v>
       </c>
@@ -6397,7 +6389,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>66</v>
       </c>
@@ -6462,7 +6454,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>67</v>
       </c>
@@ -6527,7 +6519,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>69</v>
       </c>
@@ -6592,7 +6584,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>70</v>
       </c>
@@ -6657,7 +6649,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="55" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>71</v>
       </c>
@@ -6722,7 +6714,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>72</v>
       </c>
@@ -6787,7 +6779,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>73</v>
       </c>
@@ -6852,7 +6844,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>74</v>
       </c>
@@ -6917,7 +6909,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>75</v>
       </c>
@@ -6982,7 +6974,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>76</v>
       </c>
@@ -7047,7 +7039,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>78</v>
       </c>
@@ -7112,7 +7104,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>79</v>
       </c>
@@ -7177,7 +7169,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:19" ht="165" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" ht="165" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>80</v>
       </c>
@@ -7242,7 +7234,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>81</v>
       </c>
@@ -7307,7 +7299,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>82</v>
       </c>
@@ -7372,7 +7364,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>83</v>
       </c>
@@ -7437,7 +7429,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>84</v>
       </c>
@@ -7502,7 +7494,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>85</v>
       </c>
@@ -7567,7 +7559,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:19" ht="135" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" ht="135" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>87</v>
       </c>
@@ -7632,7 +7624,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="70" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>88</v>
       </c>
@@ -7697,7 +7689,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="71" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>89</v>
       </c>
@@ -7762,7 +7754,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>90</v>
       </c>
@@ -7827,7 +7819,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>91</v>
       </c>
@@ -7892,7 +7884,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="74" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>92</v>
       </c>
@@ -7957,7 +7949,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>93</v>
       </c>
@@ -8022,7 +8014,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="76" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>94</v>
       </c>
@@ -8087,7 +8079,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>95</v>
       </c>
@@ -8152,7 +8144,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>97</v>
       </c>
@@ -8217,7 +8209,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="79" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>98</v>
       </c>
@@ -8282,7 +8274,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="80" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>99</v>
       </c>
@@ -8347,7 +8339,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>100</v>
       </c>
@@ -8412,7 +8404,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>102</v>
       </c>
@@ -8477,7 +8469,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="83" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>104</v>
       </c>
@@ -8542,7 +8534,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>105</v>
       </c>
@@ -8607,7 +8599,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:19" ht="180" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" ht="180" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>107</v>
       </c>
@@ -8672,7 +8664,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>108</v>
       </c>
@@ -8737,7 +8729,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>109</v>
       </c>
@@ -8802,7 +8794,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="88" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>112</v>
       </c>
@@ -8867,7 +8859,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="89" spans="1:19" ht="135" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" ht="135" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>114</v>
       </c>
@@ -8932,7 +8924,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="90" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>115</v>
       </c>
@@ -8997,7 +8989,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>116</v>
       </c>
@@ -9062,7 +9054,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>117</v>
       </c>
@@ -9127,7 +9119,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="93" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>118</v>
       </c>
@@ -9192,7 +9184,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>119</v>
       </c>
@@ -9257,7 +9249,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>120</v>
       </c>
@@ -9322,7 +9314,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="96" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>121</v>
       </c>
@@ -9387,7 +9379,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="97" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>122</v>
       </c>
@@ -9452,7 +9444,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="98" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>124</v>
       </c>
@@ -9517,7 +9509,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>126</v>
       </c>
@@ -9582,7 +9574,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>127</v>
       </c>
@@ -9647,7 +9639,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>128</v>
       </c>
@@ -9712,7 +9704,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="102" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>129</v>
       </c>
@@ -9777,7 +9769,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="103" spans="1:19" ht="135" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" ht="135" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>130</v>
       </c>
@@ -9842,7 +9834,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="104" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>134</v>
       </c>
@@ -9907,7 +9899,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>135</v>
       </c>
@@ -9972,7 +9964,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="106" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>136</v>
       </c>
@@ -10037,7 +10029,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>137</v>
       </c>
@@ -10102,7 +10094,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="108" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>138</v>
       </c>
@@ -10167,7 +10159,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="109" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>139</v>
       </c>
@@ -10232,7 +10224,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="110" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>140</v>
       </c>
@@ -10297,7 +10289,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="111" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>141</v>
       </c>
@@ -10362,7 +10354,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>142</v>
       </c>
@@ -10427,7 +10419,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="113" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>143</v>
       </c>
@@ -10492,7 +10484,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="114" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
         <v>144</v>
       </c>
@@ -10557,7 +10549,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="115" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>145</v>
       </c>
@@ -10622,7 +10614,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="116" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
         <v>146</v>
       </c>
@@ -10687,7 +10679,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="117" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>147</v>
       </c>
@@ -10752,7 +10744,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="118" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
         <v>148</v>
       </c>
@@ -10817,7 +10809,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="119" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
         <v>149</v>
       </c>
@@ -10882,7 +10874,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="120" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
         <v>150</v>
       </c>
@@ -10947,7 +10939,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="121" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>151</v>
       </c>
@@ -11012,7 +11004,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="122" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
         <v>152</v>
       </c>
@@ -11077,7 +11069,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="123" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>153</v>
       </c>
@@ -11142,7 +11134,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="124" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A124" s="3">
         <v>154</v>
       </c>
@@ -11208,110 +11200,104 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M124" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="Focus Work"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:M124" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="5" type="noConversion"/>
+  <conditionalFormatting sqref="B1:B108">
+    <cfRule type="duplicateValues" dxfId="38" priority="45"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B4">
-    <cfRule type="duplicateValues" dxfId="38" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="37" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="36" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="35" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31">
-    <cfRule type="duplicateValues" dxfId="34" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="33" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33">
-    <cfRule type="duplicateValues" dxfId="32" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B36:B39">
-    <cfRule type="duplicateValues" dxfId="31" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="duplicateValues" dxfId="30" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44">
-    <cfRule type="duplicateValues" dxfId="29" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B45">
-    <cfRule type="duplicateValues" dxfId="28" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46">
-    <cfRule type="duplicateValues" dxfId="27" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B71">
-    <cfRule type="duplicateValues" dxfId="26" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93">
-    <cfRule type="duplicateValues" dxfId="25" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B94">
-    <cfRule type="duplicateValues" dxfId="24" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B109:B113 B116:B1048576">
-    <cfRule type="duplicateValues" dxfId="23" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5">
-    <cfRule type="duplicateValues" dxfId="22" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F34">
-    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F46">
-    <cfRule type="duplicateValues" dxfId="20" priority="20"/>
     <cfRule type="duplicateValues" dxfId="19" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F70">
-    <cfRule type="duplicateValues" dxfId="18" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F78">
-    <cfRule type="duplicateValues" dxfId="17" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F84">
-    <cfRule type="duplicateValues" dxfId="16" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F97">
-    <cfRule type="duplicateValues" dxfId="15" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J15">
-    <cfRule type="duplicateValues" dxfId="14" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J33">
-    <cfRule type="duplicateValues" dxfId="12" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J45">
-    <cfRule type="duplicateValues" dxfId="10" priority="16"/>
     <cfRule type="duplicateValues" dxfId="9" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J61">
-    <cfRule type="duplicateValues" dxfId="8" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J66">
-    <cfRule type="duplicateValues" dxfId="6" priority="10"/>
     <cfRule type="duplicateValues" dxfId="5" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J103">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
     <cfRule type="duplicateValues" dxfId="3" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1:B108">
-    <cfRule type="duplicateValues" dxfId="0" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -13588,8 +13574,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A19">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated metrics (forgot to commit earlier)
</commit_message>
<xml_diff>
--- a/metrics and parser/DevEx_Metrics.xlsx
+++ b/metrics and parser/DevEx_Metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\DEV\UZH\DX-Metrics-Compass\metrics and parser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDDA6B45-D2A6-4EDA-9DC5-A47702197CFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ABB7680-23B3-4D06-92B1-D5AE3E75C3CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="39750" windowHeight="23385" tabRatio="506" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="39750" windowHeight="23385" tabRatio="506" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metrics" sheetId="1" r:id="rId1"/>
@@ -2514,7 +2514,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -2565,11 +2565,9 @@
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -12585,7 +12583,7 @@
       <c r="C67" t="s">
         <v>685</v>
       </c>
-      <c r="D67" s="21" t="s">
+      <c r="D67" s="20" t="s">
         <v>734</v>
       </c>
     </row>
@@ -13677,7 +13675,7 @@
       <c r="C145" t="s">
         <v>676</v>
       </c>
-      <c r="D145" s="20" t="s">
+      <c r="D145" s="19" t="s">
         <v>757</v>
       </c>
     </row>
@@ -13691,7 +13689,7 @@
       <c r="C146" t="s">
         <v>685</v>
       </c>
-      <c r="D146" s="22" t="s">
+      <c r="D146" s="19" t="s">
         <v>761</v>
       </c>
     </row>
@@ -13703,11 +13701,9 @@
   </autoFilter>
   <hyperlinks>
     <hyperlink ref="D67" r:id="rId1" xr:uid="{59EFEB55-B7A4-4807-A75B-EA48D4BA0ABA}"/>
-    <hyperlink ref="D145" r:id="rId2" xr:uid="{D917F0D9-8FA3-42FC-8D59-6D5DA7D992BF}"/>
-    <hyperlink ref="D146" r:id="rId3" xr:uid="{4212A9B2-9B1D-41C8-8E67-D931B1DC9F17}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">

</xml_diff>

<commit_message>
added "Number of Customer-Reported Defects" metric
refined subcategories with overlapping naming
fixed bug with Linkedin Framework
changed coloring of sunburst (extracted to dashboard instead of databse)
</commit_message>
<xml_diff>
--- a/metrics and parser/DevEx_Metrics.xlsx
+++ b/metrics and parser/DevEx_Metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\DEV\UZH\DX-Metrics-Compass\metrics and parser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F6DB41B-B7DB-4BEA-8598-580486DF1DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2C50DE-D839-4259-8AFB-2BC056542F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4543" yWindow="13611" windowWidth="24891" windowHeight="14915" tabRatio="506" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="23385" tabRatio="506" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metrics" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2040" uniqueCount="848">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2041" uniqueCount="850">
   <si>
     <t>id</t>
   </si>
@@ -2118,9 +2118,6 @@
     <t>Measures the time, in seconds, developers spend waiting for their builds to finish locally during development. Impacts developer flow and productivity. Considered e.g. as median (P50) or P90.</t>
   </si>
   <si>
-    <t>50; 234; 131; 146; 521</t>
-  </si>
-  <si>
     <t>501; 521</t>
   </si>
   <si>
@@ -2271,9 +2268,6 @@
     <t>Monitors AI being built into products, not just used by developer throughout the SLDC.</t>
   </si>
   <si>
-    <t>501g; 521; 510</t>
-  </si>
-  <si>
     <t>501b; 501a; 131k; 131j</t>
   </si>
   <si>
@@ -2590,6 +2584,18 @@
   </si>
   <si>
     <t>CSAT; DSAT; NSAT; Satisfaction Score; Developer Sentiment; Developer Satisfaction; Employee satisfaction; Net User Satisfaction; Satisfaction with Engineering System; Platform and Tool Satisfaction; AI tool CSAT</t>
+  </si>
+  <si>
+    <t>501g; 510</t>
+  </si>
+  <si>
+    <t>Produced Output</t>
+  </si>
+  <si>
+    <t>Product Quality</t>
+  </si>
+  <si>
+    <t>Review Process</t>
   </si>
 </sst>
 </file>
@@ -3470,6 +3476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:S123"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3549,7 +3556,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2</v>
       </c>
@@ -3614,7 +3621,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>4</v>
       </c>
@@ -3679,7 +3686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>9</v>
       </c>
@@ -3744,12 +3751,12 @@
         <v>604</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>9</v>
@@ -3758,7 +3765,7 @@
         <v>300</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>25</v>
@@ -3809,7 +3816,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>11</v>
       </c>
@@ -3874,7 +3881,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>12</v>
       </c>
@@ -3936,10 +3943,10 @@
         <v>517</v>
       </c>
       <c r="S7" s="12" t="s">
-        <v>708</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>13</v>
       </c>
@@ -3950,7 +3957,7 @@
         <v>9</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="E8" s="13" t="s">
         <v>686</v>
@@ -4004,7 +4011,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>14</v>
       </c>
@@ -4015,10 +4022,10 @@
         <v>9</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>741</v>
+        <v>846</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>37</v>
@@ -4046,7 +4053,7 @@
       </c>
       <c r="M9" s="3">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N9" s="3">
         <f t="shared" si="1"/>
@@ -4054,7 +4061,7 @@
       </c>
       <c r="O9" s="3">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="P9" s="12" t="s">
         <v>440</v>
@@ -4069,7 +4076,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>15</v>
       </c>
@@ -4083,7 +4090,7 @@
         <v>612</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>615</v>
@@ -4134,7 +4141,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>16</v>
       </c>
@@ -4204,16 +4211,16 @@
         <v>17</v>
       </c>
       <c r="B12" s="18" t="s">
+        <v>695</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>696</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>697</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>578</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>41</v>
@@ -4229,7 +4236,7 @@
         <v>206</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>15</v>
+        <v>849</v>
       </c>
       <c r="K12" s="3">
         <f>VLOOKUP(J12,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -4264,7 +4271,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>18</v>
       </c>
@@ -4329,7 +4336,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>19</v>
       </c>
@@ -4337,7 +4344,7 @@
         <v>45</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>649</v>
@@ -4346,7 +4353,7 @@
         <v>648</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>522</v>
@@ -4359,7 +4366,7 @@
         <v>207</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>46</v>
+        <v>847</v>
       </c>
       <c r="K14" s="3">
         <f>VLOOKUP(J14,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -4394,12 +4401,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>20</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>162</v>
@@ -4411,7 +4418,7 @@
         <v>584</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>521</v>
@@ -4459,12 +4466,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>22</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>9</v>
@@ -4524,12 +4531,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>23</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>163</v>
@@ -4541,7 +4548,7 @@
         <v>289</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>522</v>
@@ -4586,10 +4593,10 @@
         <v>516</v>
       </c>
       <c r="S17" s="12" t="s">
-        <v>784</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>24</v>
       </c>
@@ -4654,15 +4661,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>25</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>9</v>
@@ -4684,7 +4691,7 @@
         <v>208</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>30</v>
+        <v>848</v>
       </c>
       <c r="K19" s="3">
         <f>VLOOKUP(J19,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -4719,12 +4726,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>26</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>623</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>9</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>308</v>
@@ -4746,7 +4756,7 @@
         <v>208</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>30</v>
+        <v>848</v>
       </c>
       <c r="K20" s="3">
         <f>VLOOKUP(J20,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -4778,10 +4788,10 @@
         <v>517</v>
       </c>
       <c r="S20" s="12" t="s">
-        <v>795</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>27</v>
       </c>
@@ -4846,24 +4856,24 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>29</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>790</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>791</v>
+      </c>
+      <c r="F22" s="4" t="s">
         <v>792</v>
-      </c>
-      <c r="D22" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E22" s="13" t="s">
-        <v>793</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>794</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>522</v>
@@ -4911,7 +4921,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>30</v>
       </c>
@@ -4976,7 +4986,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>31</v>
       </c>
@@ -4984,16 +4994,16 @@
         <v>60</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="D24" s="12">
         <v>170</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="F24" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>522</v>
@@ -5038,15 +5048,15 @@
         <v>517</v>
       </c>
       <c r="S24" s="12" t="s">
-        <v>707</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>32</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>9</v>
@@ -5106,7 +5116,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>33</v>
       </c>
@@ -5171,7 +5181,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>34</v>
       </c>
@@ -5179,13 +5189,13 @@
         <v>67</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="D27" s="13" t="s">
         <v>378</v>
       </c>
       <c r="E27" s="13" t="s">
-        <v>690</v>
+        <v>302</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>689</v>
@@ -5217,11 +5227,11 @@
       </c>
       <c r="N27" s="3">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O27" s="3">
         <f t="shared" si="2"/>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="P27" s="12" t="s">
         <v>440</v>
@@ -5236,7 +5246,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>36</v>
       </c>
@@ -5244,13 +5254,13 @@
         <v>69</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>70</v>
@@ -5298,15 +5308,15 @@
         <v>517</v>
       </c>
       <c r="S28" s="12" t="s">
-        <v>832</v>
-      </c>
-    </row>
-    <row r="29" spans="1:19" ht="165" x14ac:dyDescent="0.25">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" ht="165" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>37</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>9</v>
@@ -5366,7 +5376,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>38</v>
       </c>
@@ -5374,7 +5384,7 @@
         <v>73</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>473</v>
@@ -5431,7 +5441,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>39</v>
       </c>
@@ -5496,7 +5506,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>40</v>
       </c>
@@ -5510,7 +5520,7 @@
         <v>374</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>77</v>
@@ -5561,7 +5571,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>41</v>
       </c>
@@ -5626,7 +5636,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>42</v>
       </c>
@@ -5634,13 +5644,13 @@
         <v>80</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="D34" s="12" t="s">
         <v>9</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>81</v>
@@ -5688,10 +5698,10 @@
         <v>517</v>
       </c>
       <c r="S34" s="12" t="s">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="35" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>43</v>
       </c>
@@ -5756,7 +5766,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>44</v>
       </c>
@@ -5764,10 +5774,10 @@
         <v>85</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="E36" s="13" t="s">
         <v>379</v>
@@ -5821,7 +5831,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>45</v>
       </c>
@@ -5886,15 +5896,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>46</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="D38" s="12" t="s">
         <v>9</v>
@@ -5903,7 +5913,7 @@
         <v>317</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>522</v>
@@ -5951,7 +5961,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>50</v>
       </c>
@@ -6016,7 +6026,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>56</v>
       </c>
@@ -6081,7 +6091,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>57</v>
       </c>
@@ -6146,7 +6156,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="210" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" ht="210" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>58</v>
       </c>
@@ -6211,15 +6221,15 @@
         <v>563</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>59</v>
       </c>
       <c r="B43" s="3" t="s">
+        <v>717</v>
+      </c>
+      <c r="C43" s="4" t="s">
         <v>718</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>719</v>
       </c>
       <c r="D43" s="12" t="s">
         <v>9</v>
@@ -6276,7 +6286,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>62</v>
       </c>
@@ -6284,13 +6294,13 @@
         <v>594</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>595</v>
@@ -6341,7 +6351,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>63</v>
       </c>
@@ -6406,7 +6416,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>64</v>
       </c>
@@ -6423,7 +6433,7 @@
         <v>9</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>522</v>
@@ -6471,7 +6481,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>65</v>
       </c>
@@ -6479,7 +6489,7 @@
         <v>104</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="D47" s="13" t="s">
         <v>466</v>
@@ -6536,7 +6546,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>67</v>
       </c>
@@ -6601,7 +6611,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>69</v>
       </c>
@@ -6609,7 +6619,7 @@
         <v>107</v>
       </c>
       <c r="C49" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="D49" s="12" t="s">
         <v>293</v>
@@ -6666,7 +6676,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>70</v>
       </c>
@@ -6674,13 +6684,13 @@
         <v>109</v>
       </c>
       <c r="C50" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>784</v>
+      </c>
+      <c r="E50" s="13" t="s">
         <v>785</v>
-      </c>
-      <c r="D50" s="12" t="s">
-        <v>786</v>
-      </c>
-      <c r="E50" s="13" t="s">
-        <v>787</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>629</v>
@@ -6728,10 +6738,10 @@
         <v>517</v>
       </c>
       <c r="S50" s="12" t="s">
-        <v>788</v>
-      </c>
-    </row>
-    <row r="51" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="51" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>71</v>
       </c>
@@ -6796,7 +6806,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>72</v>
       </c>
@@ -6861,7 +6871,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="53" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>73</v>
       </c>
@@ -6926,12 +6936,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>75</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>631</v>
@@ -6988,15 +6998,15 @@
         <v>518</v>
       </c>
       <c r="S54" s="12" t="s">
-        <v>732</v>
-      </c>
-    </row>
-    <row r="55" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="55" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>76</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="D55" s="12" t="s">
         <v>9</v>
@@ -7053,7 +7063,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>78</v>
       </c>
@@ -7118,7 +7128,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>79</v>
       </c>
@@ -7183,7 +7193,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>80</v>
       </c>
@@ -7213,7 +7223,7 @@
         <v>208</v>
       </c>
       <c r="J58" s="3" t="s">
-        <v>30</v>
+        <v>848</v>
       </c>
       <c r="K58" s="3">
         <f>VLOOKUP(J58,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -7248,12 +7258,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>82</v>
       </c>
       <c r="B59" s="18" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>120</v>
@@ -7313,7 +7323,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>83</v>
       </c>
@@ -7378,7 +7388,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="61" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>87</v>
       </c>
@@ -7392,7 +7402,7 @@
         <v>579</v>
       </c>
       <c r="E61" s="13" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>603</v>
@@ -7443,15 +7453,15 @@
         <v>605</v>
       </c>
     </row>
-    <row r="62" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>88</v>
       </c>
       <c r="B62" s="3" t="s">
+        <v>723</v>
+      </c>
+      <c r="C62" s="4" t="s">
         <v>724</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>725</v>
       </c>
       <c r="D62" s="10" t="s">
         <v>581</v>
@@ -7460,7 +7470,7 @@
         <v>288</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="G62" s="3" t="s">
         <v>522</v>
@@ -7508,7 +7518,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>89</v>
       </c>
@@ -7573,7 +7583,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>90</v>
       </c>
@@ -7587,10 +7597,10 @@
         <v>463</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="G64" s="3" t="s">
         <v>521</v>
@@ -7638,7 +7648,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>91</v>
       </c>
@@ -7703,7 +7713,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>92</v>
       </c>
@@ -7768,7 +7778,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>93</v>
       </c>
@@ -7833,7 +7843,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>94</v>
       </c>
@@ -7898,15 +7908,15 @@
         <v>627</v>
       </c>
     </row>
-    <row r="69" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>95</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="D69" s="13" t="s">
         <v>361</v>
@@ -7915,7 +7925,7 @@
         <v>9</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="G69" s="3" t="s">
         <v>525</v>
@@ -7960,10 +7970,10 @@
         <v>516</v>
       </c>
       <c r="S69" s="12" t="s">
-        <v>743</v>
-      </c>
-    </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="70" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>97</v>
       </c>
@@ -8028,12 +8038,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="71" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>98</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="C71" s="4" t="s">
         <v>168</v>
@@ -8093,12 +8103,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>99</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="C72" s="4" t="s">
         <v>9</v>
@@ -8110,7 +8120,7 @@
         <v>508</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="G72" s="3" t="s">
         <v>522</v>
@@ -8158,7 +8168,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>100</v>
       </c>
@@ -8223,7 +8233,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="74" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>102</v>
       </c>
@@ -8288,12 +8298,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>104</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>9</v>
@@ -8353,7 +8363,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="76" spans="1:19" ht="120" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>107</v>
       </c>
@@ -8367,7 +8377,7 @@
         <v>375</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="F76" s="4" t="s">
         <v>142</v>
@@ -8418,7 +8428,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>108</v>
       </c>
@@ -8483,24 +8493,24 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>109</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="E78" s="13" t="s">
         <v>311</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="G78" s="3" t="s">
         <v>522</v>
@@ -8545,10 +8555,10 @@
         <v>517</v>
       </c>
       <c r="S78" s="12" t="s">
-        <v>745</v>
-      </c>
-    </row>
-    <row r="79" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="79" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>112</v>
       </c>
@@ -8562,10 +8572,10 @@
         <v>9</v>
       </c>
       <c r="E79" s="13" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="F79" s="5" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="G79" s="3" t="s">
         <v>521</v>
@@ -8610,15 +8620,15 @@
         <v>518</v>
       </c>
       <c r="S79" s="12" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="80" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="80" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>113</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>491</v>
@@ -8630,7 +8640,7 @@
         <v>479</v>
       </c>
       <c r="F80" s="5" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="G80" s="3" t="s">
         <v>522</v>
@@ -8675,10 +8685,10 @@
         <v>516</v>
       </c>
       <c r="S80" s="12" t="s">
-        <v>751</v>
-      </c>
-    </row>
-    <row r="81" spans="1:19" ht="150" x14ac:dyDescent="0.25">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="81" spans="1:19" ht="150" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>114</v>
       </c>
@@ -8686,7 +8696,7 @@
         <v>630</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="D81" s="13" t="s">
         <v>652</v>
@@ -8695,7 +8705,7 @@
         <v>651</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="G81" s="3" t="s">
         <v>522</v>
@@ -8708,7 +8718,7 @@
         <v>207</v>
       </c>
       <c r="J81" s="3" t="s">
-        <v>46</v>
+        <v>847</v>
       </c>
       <c r="K81" s="3">
         <f>VLOOKUP(J81,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -8743,7 +8753,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>115</v>
       </c>
@@ -8751,7 +8761,7 @@
         <v>146</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="D82" s="12" t="s">
         <v>9</v>
@@ -8760,7 +8770,7 @@
         <v>183</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="G82" s="3" t="s">
         <v>525</v>
@@ -8805,10 +8815,10 @@
         <v>518</v>
       </c>
       <c r="S82" s="12" t="s">
-        <v>758</v>
-      </c>
-    </row>
-    <row r="83" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="83" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>116</v>
       </c>
@@ -8816,7 +8826,7 @@
         <v>147</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="D83" s="12" t="s">
         <v>576</v>
@@ -8873,7 +8883,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>117</v>
       </c>
@@ -8881,10 +8891,10 @@
         <v>35</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="D84" s="12" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="E84" s="13" t="s">
         <v>313</v>
@@ -8938,7 +8948,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>118</v>
       </c>
@@ -9003,15 +9013,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>120</v>
       </c>
       <c r="B86" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="D86" s="12" t="s">
         <v>300</v>
@@ -9020,7 +9030,7 @@
         <v>302</v>
       </c>
       <c r="F86" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="G86" s="3" t="s">
         <v>522</v>
@@ -9065,10 +9075,10 @@
         <v>516</v>
       </c>
       <c r="S86" s="12" t="s">
-        <v>765</v>
-      </c>
-    </row>
-    <row r="87" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="87" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>121</v>
       </c>
@@ -9133,7 +9143,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="88" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>122</v>
       </c>
@@ -9141,7 +9151,7 @@
         <v>156</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="D88" s="12" t="s">
         <v>653</v>
@@ -9150,7 +9160,7 @@
         <v>654</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="G88" s="3" t="s">
         <v>522</v>
@@ -9195,10 +9205,10 @@
         <v>516</v>
       </c>
       <c r="S88" s="12" t="s">
-        <v>767</v>
-      </c>
-    </row>
-    <row r="89" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="89" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>124</v>
       </c>
@@ -9263,12 +9273,12 @@
         <v>618</v>
       </c>
     </row>
-    <row r="90" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>126</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>588</v>
@@ -9293,7 +9303,7 @@
         <v>207</v>
       </c>
       <c r="J90" s="3" t="s">
-        <v>46</v>
+        <v>847</v>
       </c>
       <c r="K90" s="3">
         <f>VLOOKUP(J90,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -9328,15 +9338,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>127</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="D91" s="12" t="s">
         <v>580</v>
@@ -9358,7 +9368,7 @@
         <v>207</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>46</v>
+        <v>847</v>
       </c>
       <c r="K91" s="3">
         <f>VLOOKUP(J91,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -9390,18 +9400,18 @@
         <v>517</v>
       </c>
       <c r="S91" s="12" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="92" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="92" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>128</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="D92" s="12" t="s">
         <v>301</v>
@@ -9423,7 +9433,7 @@
         <v>207</v>
       </c>
       <c r="J92" s="3" t="s">
-        <v>46</v>
+        <v>847</v>
       </c>
       <c r="K92" s="3">
         <f>VLOOKUP(J92,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -9458,7 +9468,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="93" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>129</v>
       </c>
@@ -9466,7 +9476,7 @@
         <v>457</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="D93" s="12" t="s">
         <v>458</v>
@@ -9488,7 +9498,7 @@
         <v>207</v>
       </c>
       <c r="J93" s="3" t="s">
-        <v>46</v>
+        <v>847</v>
       </c>
       <c r="K93" s="3">
         <f>VLOOKUP(J93,cardsort_subgroup_IDs!A:B,2,0)</f>
@@ -9523,7 +9533,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>130</v>
       </c>
@@ -9531,7 +9541,7 @@
         <v>591</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="D94" s="12" t="s">
         <v>376</v>
@@ -9540,7 +9550,7 @@
         <v>377</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="G94" s="3" t="s">
         <v>521</v>
@@ -9588,24 +9598,24 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>133</v>
       </c>
       <c r="B95" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>774</v>
+      </c>
+      <c r="D95" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E95" s="13" t="s">
         <v>775</v>
       </c>
-      <c r="C95" s="4" t="s">
+      <c r="F95" s="4" t="s">
         <v>776</v>
-      </c>
-      <c r="D95" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E95" s="13" t="s">
-        <v>777</v>
-      </c>
-      <c r="F95" s="4" t="s">
-        <v>778</v>
       </c>
       <c r="G95" s="3" t="s">
         <v>522</v>
@@ -9650,27 +9660,27 @@
         <v>516</v>
       </c>
       <c r="S95" t="s">
-        <v>779</v>
-      </c>
-    </row>
-    <row r="96" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="96" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>134</v>
       </c>
       <c r="B96" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D96" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E96" s="13" t="s">
+        <v>780</v>
+      </c>
+      <c r="F96" s="4" t="s">
         <v>781</v>
-      </c>
-      <c r="C96" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D96" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E96" s="13" t="s">
-        <v>782</v>
-      </c>
-      <c r="F96" s="4" t="s">
-        <v>783</v>
       </c>
       <c r="G96" s="3" t="s">
         <v>522</v>
@@ -9715,10 +9725,10 @@
         <v>517</v>
       </c>
       <c r="S96" t="s">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="97" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="97" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>135</v>
       </c>
@@ -9783,7 +9793,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="98" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>137</v>
       </c>
@@ -9848,15 +9858,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>138</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="D99" s="12" t="s">
         <v>9</v>
@@ -9913,7 +9923,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>139</v>
       </c>
@@ -9978,7 +9988,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>140</v>
       </c>
@@ -9986,7 +9996,7 @@
         <v>432</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="D101" s="12" t="s">
         <v>454</v>
@@ -10043,12 +10053,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>141</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="C102" s="3" t="s">
         <v>660</v>
@@ -10108,12 +10118,12 @@
         <v>129</v>
       </c>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>142</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="C103" s="3" t="s">
         <v>661</v>
@@ -10173,15 +10183,15 @@
         <v>19</v>
       </c>
     </row>
-    <row r="104" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>143</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="D104" s="12" t="s">
         <v>443</v>
@@ -10190,7 +10200,7 @@
         <v>9</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="G104" s="3" t="s">
         <v>522</v>
@@ -10238,12 +10248,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>144</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>9</v>
@@ -10303,15 +10313,15 @@
         <v>448</v>
       </c>
     </row>
-    <row r="106" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>145</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="D106" s="10" t="s">
         <v>424</v>
@@ -10368,7 +10378,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="107" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>146</v>
       </c>
@@ -10376,7 +10386,7 @@
         <v>445</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="D107" t="s">
         <v>449</v>
@@ -10433,15 +10443,15 @@
         <v>450</v>
       </c>
     </row>
-    <row r="108" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>147</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="D108" s="10" t="s">
         <v>452</v>
@@ -10450,7 +10460,7 @@
         <v>9</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="G108" s="3" t="s">
         <v>522</v>
@@ -10498,12 +10508,12 @@
         <v>448</v>
       </c>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>148</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="C109" s="4" t="s">
         <v>484</v>
@@ -10563,15 +10573,15 @@
         <v>456</v>
       </c>
     </row>
-    <row r="110" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>149</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="D110" s="12" t="s">
         <v>470</v>
@@ -10580,7 +10590,7 @@
         <v>479</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="G110" s="3" t="s">
         <v>521</v>
@@ -10628,24 +10638,24 @@
         <v>464</v>
       </c>
     </row>
-    <row r="111" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>150</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="D111" s="12" t="s">
         <v>583</v>
       </c>
       <c r="E111" s="13" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="G111" s="3" t="s">
         <v>521</v>
@@ -10693,7 +10703,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>151</v>
       </c>
@@ -10758,7 +10768,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>152</v>
       </c>
@@ -10823,12 +10833,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="114" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
         <v>153</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="C114" s="4" t="s">
         <v>9</v>
@@ -10888,15 +10898,15 @@
         <v>489</v>
       </c>
     </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>154</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="D115" s="12" t="s">
         <v>9</v>
@@ -10905,7 +10915,7 @@
         <v>485</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="G115" s="3" t="s">
         <v>521</v>
@@ -10953,7 +10963,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="116" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
         <v>155</v>
       </c>
@@ -11015,10 +11025,10 @@
         <v>516</v>
       </c>
       <c r="S116" s="12" t="s">
-        <v>710</v>
-      </c>
-    </row>
-    <row r="117" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="117" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>156</v>
       </c>
@@ -11083,7 +11093,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
         <v>157</v>
       </c>
@@ -11148,15 +11158,15 @@
         <v>564</v>
       </c>
     </row>
-    <row r="119" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
         <v>158</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="D119" s="12" t="s">
         <v>9</v>
@@ -11165,7 +11175,7 @@
         <v>505</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="G119" s="3" t="s">
         <v>522</v>
@@ -11213,7 +11223,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="120" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
         <v>159</v>
       </c>
@@ -11278,7 +11288,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="121" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>160</v>
       </c>
@@ -11343,7 +11353,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="122" spans="1:19" ht="45" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
         <v>161</v>
       </c>
@@ -11408,24 +11418,24 @@
         <v>683</v>
       </c>
     </row>
-    <row r="123" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>162</v>
       </c>
       <c r="B123" s="3" t="s">
+        <v>831</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D123" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E123" s="13" t="s">
+        <v>832</v>
+      </c>
+      <c r="F123" s="4" t="s">
         <v>833</v>
-      </c>
-      <c r="C123" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D123" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="E123" s="13" t="s">
-        <v>834</v>
-      </c>
-      <c r="F123" s="4" t="s">
-        <v>835</v>
       </c>
       <c r="G123" s="3" t="s">
         <v>522</v>
@@ -11467,14 +11477,20 @@
         <v>511</v>
       </c>
       <c r="R123" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="S123" s="12" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M123" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:M123" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="Process"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="B4">
     <cfRule type="duplicateValues" dxfId="41" priority="30"/>
@@ -13700,16 +13716,16 @@
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="10" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="B151" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="C151" t="s">
         <v>504</v>
       </c>
       <c r="D151" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
     </row>
   </sheetData>
@@ -13906,7 +13922,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>15</v>
+        <v>849</v>
       </c>
       <c r="B11">
         <v>311</v>
@@ -13914,7 +13930,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>46</v>
+        <v>847</v>
       </c>
       <c r="B12">
         <v>312</v>
@@ -13946,7 +13962,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>30</v>
+        <v>848</v>
       </c>
       <c r="B16">
         <v>317</v>

</xml_diff>

<commit_message>
[#5] Add "report a metric" form and supporting API
Users can now report missing metrics (via footer link or thumbs-down
feedback) or flag an issue with an existing metric (via the tooltip
button). Reports are POSTed to a new api/ folder with shared PHP
helpers covering origin checks, rate limiting, IP anonymisation, and
log protection via .htaccess.

Also: clearing the shortlist resets the step-1 entry panel; feedback.php
moved to api/ alongside the new endpoint.
</commit_message>
<xml_diff>
--- a/metrics and parser/DevEx_Metrics.xlsx
+++ b/metrics and parser/DevEx_Metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\DEV\UZH\DX-Metrics-Compass\metrics and parser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2C50DE-D839-4259-8AFB-2BC056542F44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{200DC2C8-BB83-4622-89CB-B5F71CE604A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="23385" tabRatio="506" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="29010" windowHeight="23385" tabRatio="506" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metrics" sheetId="1" r:id="rId1"/>
@@ -3476,7 +3476,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:S123"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3556,7 +3555,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>2</v>
       </c>
@@ -3621,7 +3620,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="3" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>4</v>
       </c>
@@ -3686,7 +3685,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>9</v>
       </c>
@@ -3751,7 +3750,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>10</v>
       </c>
@@ -3816,7 +3815,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>11</v>
       </c>
@@ -3881,7 +3880,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>12</v>
       </c>
@@ -3946,7 +3945,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>13</v>
       </c>
@@ -4011,7 +4010,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>14</v>
       </c>
@@ -4076,7 +4075,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>15</v>
       </c>
@@ -4141,7 +4140,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>16</v>
       </c>
@@ -4271,7 +4270,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>18</v>
       </c>
@@ -4336,7 +4335,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>19</v>
       </c>
@@ -4401,7 +4400,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>20</v>
       </c>
@@ -4466,7 +4465,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>22</v>
       </c>
@@ -4531,7 +4530,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>23</v>
       </c>
@@ -4596,7 +4595,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>24</v>
       </c>
@@ -4661,7 +4660,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>25</v>
       </c>
@@ -4726,7 +4725,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="20" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>26</v>
       </c>
@@ -4791,7 +4790,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>27</v>
       </c>
@@ -4856,7 +4855,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>29</v>
       </c>
@@ -4921,7 +4920,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>30</v>
       </c>
@@ -4986,7 +4985,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="24" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>31</v>
       </c>
@@ -5051,7 +5050,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>32</v>
       </c>
@@ -5116,7 +5115,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>33</v>
       </c>
@@ -5181,7 +5180,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>34</v>
       </c>
@@ -5246,7 +5245,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>36</v>
       </c>
@@ -5311,7 +5310,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="165" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" ht="165" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>37</v>
       </c>
@@ -5376,7 +5375,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>38</v>
       </c>
@@ -5441,7 +5440,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>39</v>
       </c>
@@ -5506,7 +5505,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>40</v>
       </c>
@@ -5571,7 +5570,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>41</v>
       </c>
@@ -5636,7 +5635,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>42</v>
       </c>
@@ -5701,7 +5700,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>43</v>
       </c>
@@ -5766,7 +5765,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>44</v>
       </c>
@@ -5831,7 +5830,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>45</v>
       </c>
@@ -5896,7 +5895,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>46</v>
       </c>
@@ -5961,7 +5960,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>50</v>
       </c>
@@ -6026,7 +6025,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>56</v>
       </c>
@@ -6091,7 +6090,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>57</v>
       </c>
@@ -6156,7 +6155,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="210" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" ht="210" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>58</v>
       </c>
@@ -6221,7 +6220,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="43" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>59</v>
       </c>
@@ -6286,7 +6285,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>62</v>
       </c>
@@ -6351,7 +6350,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>63</v>
       </c>
@@ -6416,7 +6415,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>64</v>
       </c>
@@ -6481,7 +6480,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>65</v>
       </c>
@@ -6546,7 +6545,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>67</v>
       </c>
@@ -6611,7 +6610,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>69</v>
       </c>
@@ -6676,7 +6675,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="50" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>70</v>
       </c>
@@ -6741,7 +6740,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="51" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>71</v>
       </c>
@@ -6806,7 +6805,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>72</v>
       </c>
@@ -6871,7 +6870,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="53" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>73</v>
       </c>
@@ -6936,7 +6935,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>75</v>
       </c>
@@ -7001,7 +7000,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="55" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>76</v>
       </c>
@@ -7063,7 +7062,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>78</v>
       </c>
@@ -7128,7 +7127,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="57" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>79</v>
       </c>
@@ -7193,7 +7192,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>80</v>
       </c>
@@ -7258,7 +7257,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="59" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>82</v>
       </c>
@@ -7323,7 +7322,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>83</v>
       </c>
@@ -7388,7 +7387,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="61" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>87</v>
       </c>
@@ -7453,7 +7452,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="62" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>88</v>
       </c>
@@ -7518,7 +7517,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="63" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>89</v>
       </c>
@@ -7583,7 +7582,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>90</v>
       </c>
@@ -7648,7 +7647,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>91</v>
       </c>
@@ -7713,7 +7712,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>92</v>
       </c>
@@ -7778,7 +7777,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="67" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>93</v>
       </c>
@@ -7843,7 +7842,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>94</v>
       </c>
@@ -7908,7 +7907,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="69" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>95</v>
       </c>
@@ -7973,7 +7972,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="70" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>97</v>
       </c>
@@ -8038,7 +8037,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="71" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>98</v>
       </c>
@@ -8103,7 +8102,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="72" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>99</v>
       </c>
@@ -8168,7 +8167,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>100</v>
       </c>
@@ -8233,7 +8232,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="74" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>102</v>
       </c>
@@ -8298,7 +8297,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="75" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>104</v>
       </c>
@@ -8363,7 +8362,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="76" spans="1:19" ht="120" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" ht="120" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>107</v>
       </c>
@@ -8428,7 +8427,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>108</v>
       </c>
@@ -8493,7 +8492,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="78" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>109</v>
       </c>
@@ -8558,7 +8557,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="79" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>112</v>
       </c>
@@ -8623,7 +8622,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="80" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>113</v>
       </c>
@@ -8688,7 +8687,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="81" spans="1:19" ht="150" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" ht="150" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>114</v>
       </c>
@@ -8753,7 +8752,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>115</v>
       </c>
@@ -8818,7 +8817,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="83" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>116</v>
       </c>
@@ -8883,7 +8882,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>117</v>
       </c>
@@ -8948,7 +8947,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>118</v>
       </c>
@@ -9013,7 +9012,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>120</v>
       </c>
@@ -9078,7 +9077,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="87" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>121</v>
       </c>
@@ -9143,7 +9142,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="88" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>122</v>
       </c>
@@ -9208,7 +9207,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="89" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>124</v>
       </c>
@@ -9273,7 +9272,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="90" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>126</v>
       </c>
@@ -9338,7 +9337,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>127</v>
       </c>
@@ -9403,7 +9402,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="92" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>128</v>
       </c>
@@ -9468,7 +9467,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="93" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>129</v>
       </c>
@@ -9533,7 +9532,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>130</v>
       </c>
@@ -9598,7 +9597,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>133</v>
       </c>
@@ -9663,7 +9662,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="96" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>134</v>
       </c>
@@ -9728,7 +9727,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="97" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>135</v>
       </c>
@@ -9793,7 +9792,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="98" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A98" s="3">
         <v>137</v>
       </c>
@@ -9858,7 +9857,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A99" s="3">
         <v>138</v>
       </c>
@@ -9923,7 +9922,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A100" s="3">
         <v>139</v>
       </c>
@@ -9988,7 +9987,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A101" s="3">
         <v>140</v>
       </c>
@@ -10053,7 +10052,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="102" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A102" s="3">
         <v>141</v>
       </c>
@@ -10118,7 +10117,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="103" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A103" s="3">
         <v>142</v>
       </c>
@@ -10183,7 +10182,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="104" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A104" s="3">
         <v>143</v>
       </c>
@@ -10248,7 +10247,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A105" s="3">
         <v>144</v>
       </c>
@@ -10313,7 +10312,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="106" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A106" s="3">
         <v>145</v>
       </c>
@@ -10378,7 +10377,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="107" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A107" s="3">
         <v>146</v>
       </c>
@@ -10443,7 +10442,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="108" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A108" s="3">
         <v>147</v>
       </c>
@@ -10508,7 +10507,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="109" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A109" s="3">
         <v>148</v>
       </c>
@@ -10573,7 +10572,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="110" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A110" s="3">
         <v>149</v>
       </c>
@@ -10638,7 +10637,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="111" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A111" s="3">
         <v>150</v>
       </c>
@@ -10703,7 +10702,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A112" s="3">
         <v>151</v>
       </c>
@@ -10768,7 +10767,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="113" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A113" s="3">
         <v>152</v>
       </c>
@@ -10833,7 +10832,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="114" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A114" s="3">
         <v>153</v>
       </c>
@@ -10898,7 +10897,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="115" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A115" s="3">
         <v>154</v>
       </c>
@@ -10963,7 +10962,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="116" spans="1:19" ht="105" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" ht="105" x14ac:dyDescent="0.25">
       <c r="A116" s="3">
         <v>155</v>
       </c>
@@ -11028,7 +11027,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="117" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A117" s="3">
         <v>156</v>
       </c>
@@ -11093,7 +11092,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118" spans="1:19" ht="90" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:19" ht="90" x14ac:dyDescent="0.25">
       <c r="A118" s="3">
         <v>157</v>
       </c>
@@ -11158,7 +11157,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="119" spans="1:19" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:19" ht="30" x14ac:dyDescent="0.25">
       <c r="A119" s="3">
         <v>158</v>
       </c>
@@ -11223,7 +11222,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="120" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A120" s="3">
         <v>159</v>
       </c>
@@ -11288,7 +11287,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="121" spans="1:19" ht="75" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" ht="75" x14ac:dyDescent="0.25">
       <c r="A121" s="3">
         <v>160</v>
       </c>
@@ -11353,7 +11352,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="122" spans="1:19" ht="45" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A122" s="3">
         <v>161</v>
       </c>
@@ -11418,7 +11417,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="123" spans="1:19" ht="60" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A123" s="3">
         <v>162</v>
       </c>
@@ -11484,13 +11483,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M123" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="Process"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:M123" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <conditionalFormatting sqref="B4">
     <cfRule type="duplicateValues" dxfId="41" priority="30"/>

</xml_diff>